<commit_message>
Track DigiKey order and single-leg procurement gaps
</commit_message>
<xml_diff>
--- a/procurement/mode_a_procurement_bom_2026-08-21.xlsx
+++ b/procurement/mode_a_procurement_bom_2026-08-21.xlsx
@@ -2,14 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Rcc2e4065233f45e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order Now" sheetId="2" r:id="R10158225b38640b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conditional" sheetId="3" r:id="R2da7ebab228543d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ &amp; Holds" sheetId="4" r:id="Re16adbfea2b3431d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplier Carts" sheetId="5" r:id="R8d047e1048aa463e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owned &amp; Printed" sheetId="6" r:id="Rd2482823a30c4882"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" r:id="Re92507a3d2a64830"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order Links" sheetId="8" r:id="Ra5be7567d8bb4c6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R6104ca8232a44355"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order Now" sheetId="2" r:id="R2c6a12c4dcf64474"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conditional" sheetId="3" r:id="R920cfae8e15e42f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ &amp; Holds" sheetId="4" r:id="Rc338f2202a2a4427"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplier Carts" sheetId="5" r:id="Rd0c8fa95d680436f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owned &amp; Printed" sheetId="6" r:id="R917f6ba2bbd14e92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" r:id="R5cefc1164b6e4fb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order Links" sheetId="8" r:id="Rc60e9ae50ab74bdc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status &amp; Gaps" sheetId="9" r:id="R06172480efc546b4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -24,7 +25,7 @@
     <x:numFmt numFmtId="200" formatCode="$#,##0.00"/>
     <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
-  <x:fonts count="44">
+  <x:fonts count="54">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -275,8 +276,66 @@
       <x:color rgb="FF0563C1"/>
       <x:name val="Aptos"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FF173A5E"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FF217346"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FFB3261E"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF213547"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF213547"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF5F6B76"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF213547"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFB3261E"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFA65A00"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF217346"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="18">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -323,8 +382,48 @@
         <x:fgColor rgb="FFF29F3D"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE6F4EA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFCE8E6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF1F3F5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF173A5E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF008C86"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="22">
+  <x:borders count="23">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -494,11 +593,25 @@
         <x:color rgb="FFB42318"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFC9D4DE"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFC9D4DE"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFC9D4DE"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFC9D4DE"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="193">
+  <x:cellXfs count="248">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -954,11 +1067,186 @@
     <x:xf numFmtId="0" fontId="43" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="0"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="44" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="39" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="45" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="46" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="38" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="48" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="48" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="45" fillId="11" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="11" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="48" fillId="13" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="48" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="48" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="48" fillId="14" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="48" fillId="14" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="48" fillId="10" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="48" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="48" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="49" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="16" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="48" fillId="10" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="48" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="48" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="48" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="50" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="50" fillId="12" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="51" fillId="12" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="50" fillId="10" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="50" fillId="17" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="52" fillId="17" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="50" fillId="11" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="53" fillId="11" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="49" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="16" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="48" fillId="10" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="48" fillId="10" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="48" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="51" fillId="12" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="50" fillId="10" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="52" fillId="17" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="53" fillId="11" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="OrderedInTransit" displayName="OrderedInTransit" ref="A5:I9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="9">
+    <x:tableColumn id="1" name="Order date"/>
+    <x:tableColumn id="2" name="State"/>
+    <x:tableColumn id="3" name="Supplier"/>
+    <x:tableColumn id="4" name="Category"/>
+    <x:tableColumn id="5" name="Item"/>
+    <x:tableColumn id="6" name="DigiKey SKU"/>
+    <x:tableColumn id="7" name="Qty"/>
+    <x:tableColumn id="8" name="Intended use"/>
+    <x:tableColumn id="9" name="Receive &amp; verify"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="InitialBuildReadiness" displayName="InitialBuildReadiness" ref="A12:I21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="9">
+    <x:tableColumn id="1" name="Phase / gate"/>
+    <x:tableColumn id="2" name="State"/>
+    <x:tableColumn id="3" name="Item"/>
+    <x:tableColumn id="4" name="Where tracked"/>
+    <x:tableColumn id="5" name="Next action"/>
+    <x:tableColumn id="6" name="Why / compatibility"/>
+    <x:tableColumn id="7" name="Buy timing"/>
+    <x:tableColumn id="8" name="Lowest-cost path"/>
+    <x:tableColumn id="9" name="Source / evidence"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1180,7 +1468,7 @@
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
       <x:c r="A2" s="146" t="str">
-        <x:v>Los Altos, California • researched 2026-08-21 • ABS fit campaign first • all structural PA-CF and Fusion release gates preserved</x:v>
+        <x:v>Los Altos, California • procurement status updated 2026-08-31 • ABS fit campaign first • all structural PA-CF and Fusion release gates preserved</x:v>
       </x:c>
       <x:c r="B2" s="146"/>
       <x:c r="C2" s="146"/>
@@ -1202,7 +1490,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="148" t="str">
-        <x:v>BUY-NOW LIST SUBTOTAL</x:v>
+        <x:v>OPEN BUY-NOW SUBTOTAL</x:v>
       </x:c>
       <x:c r="B4" s="149"/>
       <x:c r="C4" s="147"/>
@@ -1219,7 +1507,7 @@
     <x:row r="5">
       <x:c r="A5" s="154" t="n">
         <x:f>'Order Now'!H26</x:f>
-        <x:v>181.00000000000003</x:v>
+        <x:v>146.32000000000005</x:v>
       </x:c>
       <x:c r="B5" s="155"/>
       <x:c r="C5" s="147"/>
@@ -1271,10 +1559,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B9" s="168" t="str">
-        <x:v>Order the direct electronics and standard hardware</x:v>
+        <x:v>Receive DigiKey order; buy remaining direct hardware</x:v>
       </x:c>
       <x:c r="C9" s="169" t="str">
-        <x:v>Use Order Now and Supplier Carts. The formula-linked list subtotal is the best verified pre-tax, pre-shipping number available today.</x:v>
+        <x:v>The four DigiKey line items were ordered 2026-08-31 and are tracked as in transit on Status &amp; Gaps. Use Order Now and Supplier Carts for the remaining open lines.</x:v>
       </x:c>
       <x:c r="D9" s="147"/>
       <x:c r="E9" s="147"/>
@@ -1303,10 +1591,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B11" s="168" t="str">
-        <x:v>Send the five exact RFQs now</x:v>
+        <x:v>Resolve the five exact RFQs</x:v>
       </x:c>
       <x:c r="C11" s="169" t="str">
-        <x:v>Spring, Ø10 h6 pin, Ø6 h6 pin, Ø5 h6 shaft and Ø19/13.6 shim. Early quotes can run in parallel with ABS printing.</x:v>
+        <x:v>Spring, Ø10 knee axle, Ø6 stop pin, Ø5 guide shaft and Ø19/13.6 shims. For the knee axle, do not accept a common m6 dowel; require h6 or a verified tighter h5 shaft.</x:v>
       </x:c>
       <x:c r="D11" s="147"/>
       <x:c r="E11" s="147"/>
@@ -1452,7 +1740,7 @@
     </x:row>
     <x:row r="23" ht="34" customHeight="1">
       <x:c r="A23" s="173" t="str">
-        <x:v>The buy-now subtotal is catalog/list price only. It excludes sales tax, shipping, the custom spring, precision-pin/shim quotes and anything on Conditional.</x:v>
+        <x:v>The open buy-now subtotal excludes items marked ordered/in transit or owned. It still excludes sales tax, shipping, custom precision-part quotes and anything on Conditional.</x:v>
       </x:c>
       <x:c r="B23" s="173"/>
       <x:c r="C23" s="173"/>
@@ -1498,7 +1786,7 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="174" t="str">
-        <x:v>Workbook tabs: Order Now • Conditional • RFQ &amp; Holds • Supplier Carts • Owned &amp; Printed • Sources • Order Links</x:v>
+        <x:v>Workbook tabs: Order Now • Conditional • RFQ &amp; Holds • Supplier Carts • Owned &amp; Printed • Sources • Order Links • Status &amp; Gaps</x:v>
       </x:c>
       <x:c r="B27" s="174"/>
       <x:c r="C27" s="174"/>
@@ -1573,7 +1861,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="146" t="str">
-        <x:v>One ABS fit/assembly leg plus the first safe powered bench campaign. Prices checked 2026-08-21; tax and shipping are excluded. Package quantities intentionally include working spares.</x:v>
+        <x:v>One ABS fit/assembly leg plus the first safe powered bench campaign. Status updated 2026-08-31; tax and shipping are excluded. The subtotal includes only still-open lines.</x:v>
       </x:c>
       <x:c r="B2" s="146"/>
       <x:c r="C2" s="146"/>
@@ -1667,8 +1955,7 @@
         <x:v>3.95</x:v>
       </x:c>
       <x:c r="H5" s="177" t="n">
-        <x:f>ROUND(F5*G5,2)</x:f>
-        <x:v>7.9</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I5" s="176" t="str">
         <x:v>DigiKey</x:v>
@@ -1676,14 +1963,14 @@
       <x:c r="J5" s="176" t="str">
         <x:v>1528-5708-ND</x:v>
       </x:c>
-      <x:c r="K5" s="178" t="str">
-        <x:v>URL tab →</x:v>
+      <x:c r="K5" s="194" t="str">
+        <x:v>ORDERED 2026-08-31</x:v>
       </x:c>
       <x:c r="L5" s="176" t="str">
         <x:v>With board unpowered, switch termination ON and measure CANH–CANL ≈120 Ω. Current DigiKey stock is preferred over uncertain older direct stock.</x:v>
       </x:c>
       <x:c r="M5" s="176" t="str">
-        <x:v>Consolidate with AS5048A + header.</x:v>
+        <x:v>Ordered from DigiKey 2026-08-31; receive/verify on Status &amp; Gaps.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="21.600000381469727" hidden="0" customHeight="1">
@@ -1709,8 +1996,7 @@
         <x:v>19.4</x:v>
       </x:c>
       <x:c r="H6" s="177" t="n">
-        <x:f>ROUND(F6*G6,2)</x:f>
-        <x:v>19.4</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I6" s="176" t="str">
         <x:v>DigiKey</x:v>
@@ -1718,14 +2004,14 @@
       <x:c r="J6" s="176" t="str">
         <x:v>4991-AS5048AADAPTERBOARD-ND</x:v>
       </x:c>
-      <x:c r="K6" s="178" t="str">
-        <x:v>URL tab →</x:v>
+      <x:c r="K6" s="194" t="str">
+        <x:v>ORDERED 2026-08-31</x:v>
       </x:c>
       <x:c r="L6" s="176" t="str">
         <x:v>Confirm the loose Ø6 × 2.5 mm magnet is physically in the bag before assembly.</x:v>
       </x:c>
       <x:c r="M6" s="176" t="str">
-        <x:v>Discontinued product; 335 shown in stock when checked.</x:v>
+        <x:v>Ordered from DigiKey 2026-08-31; receive/verify on Status &amp; Gaps.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="21.600000381469727" hidden="0" customHeight="1">
@@ -1751,8 +2037,7 @@
         <x:v>0.89</x:v>
       </x:c>
       <x:c r="H7" s="177" t="n">
-        <x:f>ROUND(F7*G7,2)</x:f>
-        <x:v>0.89</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I7" s="176" t="str">
         <x:v>DigiKey</x:v>
@@ -1760,14 +2045,14 @@
       <x:c r="J7" s="176" t="str">
         <x:v>609-78511-108HLF-ND</x:v>
       </x:c>
-      <x:c r="K7" s="178" t="str">
-        <x:v>URL tab →</x:v>
+      <x:c r="K7" s="194" t="str">
+        <x:v>ORDERED 2026-08-31</x:v>
       </x:c>
       <x:c r="L7" s="176" t="str">
         <x:v>Dry-fit orientation before soldering; P1 is delivered unpopulated.</x:v>
       </x:c>
       <x:c r="M7" s="176" t="str">
-        <x:v>Same DigiKey cart.</x:v>
+        <x:v>Ordered from DigiKey 2026-08-31; receive/verify on Status &amp; Gaps.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="21.600000381469727" hidden="0" customHeight="1">
@@ -2255,8 +2540,7 @@
         <x:v>6.49</x:v>
       </x:c>
       <x:c r="H19" s="177" t="n">
-        <x:f>ROUND(F19*G19,2)</x:f>
-        <x:v>6.49</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I19" s="176" t="str">
         <x:v>Walmart</x:v>
@@ -2264,14 +2548,14 @@
       <x:c r="J19" s="176" t="str">
         <x:v>6800-2RS 2-pack</x:v>
       </x:c>
-      <x:c r="K19" s="178" t="str">
-        <x:v>URL tab →</x:v>
+      <x:c r="K19" s="196" t="str">
+        <x:v>OWNED</x:v>
       </x:c>
       <x:c r="L19" s="176" t="str">
         <x:v>Confirm 10 mm bore, 19 mm OD, 5 mm width and smooth rotation.</x:v>
       </x:c>
       <x:c r="M19" s="176" t="str">
-        <x:v>Add to the Walmart PSU order if available.</x:v>
+        <x:v>Two bearings are in hand per the project README; excluded from the open subtotal.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="21.600000381469727" hidden="0" customHeight="1">
@@ -2528,7 +2812,7 @@
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
       <x:c r="A26" s="179" t="str">
-        <x:v>KNOWN DIRECT-ORDER LIST SUBTOTAL — excludes tax, shipping, RFQ items and conditional purchases</x:v>
+        <x:v>OPEN DIRECT-ORDER LIST SUBTOTAL — excludes ordered/in-transit, owned, tax, shipping, RFQ items and conditional purchases</x:v>
       </x:c>
       <x:c r="B26" s="179"/>
       <x:c r="C26" s="179"/>
@@ -2538,7 +2822,7 @@
       <x:c r="G26" s="180"/>
       <x:c r="H26" s="180" t="n">
         <x:f>SUM(H5:H25)</x:f>
-        <x:v>181.00000000000003</x:v>
+        <x:v>146.32000000000005</x:v>
       </x:c>
       <x:c r="I26" s="179"/>
       <x:c r="J26" s="179"/>
@@ -3159,8 +3443,8 @@
       </x:c>
     </x:row>
     <x:row r="6" ht="21.600000381469727" hidden="0" customHeight="1">
-      <x:c r="A6" s="183" t="str">
-        <x:v>RFQ / verify</x:v>
+      <x:c r="A6" s="198" t="str">
+        <x:v>RFQ / VERIFY — NO m6 SUBSTITUTE</x:v>
       </x:c>
       <x:c r="B6" s="176" t="str">
         <x:v>Pins</x:v>
@@ -3169,25 +3453,25 @@
         <x:v>Ø10 h6 × 35 hardened ground dowel</x:v>
       </x:c>
       <x:c r="D6" s="176" t="str">
-        <x:v>10.000 mm h6 tolerance, 35 mm length, hardened and ground</x:v>
+        <x:v>10.000/−0.009 mm (ISO h6), 35 mm finished length, hardened and ground</x:v>
       </x:c>
       <x:c r="E6" s="176" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F6" s="176" t="str">
-        <x:v>Ask WDS to certify h6 for its 10×35 precision pin; otherwise quote a custom pin.</x:v>
+        <x:v>WDS 662-20635 is catalogued as 10 × 35 mm hardened/ground at $1.31, but its page omits diameter tolerance. Ask WDS for written 9.991–10.000 mm confirmation; order only if confirmed.</x:v>
       </x:c>
       <x:c r="G6" s="178" t="str">
         <x:v>WDS Components</x:v>
       </x:c>
       <x:c r="H6" s="178" t="str">
-        <x:v>Custom fallback</x:v>
+        <x:v>MISUMI PSFU10-35: hardened SUJ2, h5 (a tighter subset of h6). Verify US availability, finished-length tolerance and usable end face before ordering.</x:v>
       </x:c>
       <x:c r="I6" s="176" t="str">
-        <x:v>The visible catalog page gives the dimensions but does not publish the required h6 tolerance.</x:v>
+        <x:v>Common DIN 6325 dowels are usually m6 (positive tolerance) and can interfere with a nominal 10 mm bearing bore. A shoulder bolt is too loose for the angular datum.</x:v>
       </x:c>
       <x:c r="J6" s="176" t="str">
-        <x:v>Supplier certificate/drawing explicitly stating h6.</x:v>
+        <x:v>Supplier certificate/drawing explicitly stating h6, or the verified MISUMI h5 drawing plus acceptable end and length finish.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="21.600000381469727" hidden="0" customHeight="1">
@@ -3353,7 +3637,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="146" t="str">
-        <x:v>The catalog subtotal is formula-linked to Order Now. Shipping is deliberately not guessed. Consolidate only exact parts; do not trade tolerance or insert length for a cheaper cart.</x:v>
+        <x:v>The open subtotal is formula-linked to Order Now and excludes ordered/in-transit and owned lines. Shipping is deliberately not guessed.</x:v>
       </x:c>
       <x:c r="B2" s="146"/>
       <x:c r="C2" s="146"/>
@@ -3399,11 +3683,11 @@
         <x:v>DigiKey</x:v>
       </x:c>
       <x:c r="B5" s="176" t="str">
-        <x:v>CAN Pal ×2; AS5048A kit; 1×8 header</x:v>
+        <x:v>CAN Pal ×2; AS5048A kit; 1×8 header — ordered 2026-08-31</x:v>
       </x:c>
       <x:c r="C5" s="177" t="n">
         <x:f>SUMIF('Order Now'!$I$5:$I$25,A5,'Order Now'!$H$5:$H$25)</x:f>
-        <x:v>28.189999999999998</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D5" s="176" t="str">
         <x:v>One electronics cart. Check termination resistors on receipt.</x:v>
@@ -3411,11 +3695,11 @@
       <x:c r="E5" s="176" t="str">
         <x:v>Normal parcel charge may apply below free-shipping threshold.</x:v>
       </x:c>
-      <x:c r="F5" s="176" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G5" s="176" t="str">
-        <x:v>Order now; AS5048A is discontinued once stock is gone.</x:v>
+      <x:c r="F5" s="194" t="str">
+        <x:v>DONE</x:v>
+      </x:c>
+      <x:c r="G5" s="194" t="str">
+        <x:v>Receive and verify on Status &amp; Gaps; do not reorder.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -3447,11 +3731,11 @@
         <x:v>Walmart</x:v>
       </x:c>
       <x:c r="B7" s="176" t="str">
-        <x:v>SPS305 PSU; 6800-2RS 2-pack</x:v>
+        <x:v>SPS305 PSU only; 6800-2RS pair is owned</x:v>
       </x:c>
       <x:c r="C7" s="177" t="n">
         <x:f>SUMIF('Order Now'!$I$5:$I$25,A7,'Order Now'!$H$5:$H$25)</x:f>
-        <x:v>45.480000000000004</x:v>
+        <x:v>38.99</x:v>
       </x:c>
       <x:c r="D7" s="176" t="str">
         <x:v>Put both lines in one cart if marketplace availability permits.</x:v>
@@ -3463,7 +3747,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G7" s="176" t="str">
-        <x:v>Order now; verify seller/returns at checkout.</x:v>
+        <x:v>Order the PSU if still missing; do not reorder bearings.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -3612,12 +3896,12 @@
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="188" t="str">
-        <x:v>LINKED LIST SUBTOTAL</x:v>
+        <x:v>OPEN LINKED LIST SUBTOTAL</x:v>
       </x:c>
       <x:c r="B14" s="188"/>
       <x:c r="C14" s="189" t="n">
         <x:f>SUM(C5:C13)</x:f>
-        <x:v>181</x:v>
+        <x:v>146.32000000000002</x:v>
       </x:c>
       <x:c r="D14" s="188"/>
       <x:c r="E14" s="188"/>
@@ -3895,22 +4179,42 @@
       </x:c>
     </x:row>
     <x:row r="15" ht="32.400001525878906" hidden="0" customHeight="1">
-      <x:c r="A15" s="190" t="str">
+      <x:c r="A15" s="205" t="str">
+        <x:v>Owned</x:v>
+      </x:c>
+      <x:c r="B15" s="206" t="str">
+        <x:v>Bearings</x:v>
+      </x:c>
+      <x:c r="C15" s="206" t="str">
+        <x:v>6800-2RS bearings</x:v>
+      </x:c>
+      <x:c r="D15" s="206" t="str">
+        <x:v>2 delivered</x:v>
+      </x:c>
+      <x:c r="E15" s="206" t="str">
+        <x:v>README.md / owner update</x:v>
+      </x:c>
+      <x:c r="F15" s="206" t="str">
+        <x:v>Use one real bearing for the indexed ABS bore-ladder test; do not force it into the failed Ø19.00 coupon.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="207" t="str">
         <x:v>Deferred</x:v>
       </x:c>
-      <x:c r="B15" s="190" t="str">
+      <x:c r="B16" s="207" t="str">
         <x:v>Mode B rail rig</x:v>
       </x:c>
-      <x:c r="C15" s="190" t="str">
+      <x:c r="C16" s="207" t="str">
         <x:v>MGN12 rail/blocks, extrusion, rail hardware, quick-release pin, PU bumpers, ballast, M12 washers, M4 studs/inserts</x:v>
       </x:c>
-      <x:c r="D15" s="190" t="str">
+      <x:c r="D16" s="207" t="str">
         <x:v>Do not buy</x:v>
       </x:c>
-      <x:c r="E15" s="190" t="str">
+      <x:c r="E16" s="207" t="str">
         <x:v>beni_single_leg_rig_design_record.md §9</x:v>
       </x:c>
-      <x:c r="F15" s="190" t="str">
+      <x:c r="F16" s="207" t="str">
         <x:v>Re-open only after Mode A fixture and measurement gates pass.</x:v>
       </x:c>
     </x:row>
@@ -4263,6 +4567,86 @@
         <x:v>Price remains TBD until drawing/spec review.</x:v>
       </x:c>
     </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="213" t="str">
+        <x:v>Current supplier</x:v>
+      </x:c>
+      <x:c r="B19" s="211" t="str">
+        <x:v>WDS 662-20635</x:v>
+      </x:c>
+      <x:c r="C19" s="211" t="str">
+        <x:v>Catalog 10 × 35 mm hardened/ground pin and current single-unit list price; diameter tolerance is not published</x:v>
+      </x:c>
+      <x:c r="D19" s="212" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="E19" s="211" t="str">
+        <x:v>https://www.wdscomponents.com/en-us/10mm-x-35mm-steel-precision-dowel-pin</x:v>
+      </x:c>
+      <x:c r="F19" s="211" t="str">
+        <x:v>Do not order until WDS confirms h6 in writing.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="213" t="str">
+        <x:v>Manufacturer</x:v>
+      </x:c>
+      <x:c r="B20" s="211" t="str">
+        <x:v>MISUMI straight linear shafts</x:v>
+      </x:c>
+      <x:c r="C20" s="211" t="str">
+        <x:v>PSFU series uses hardened SUJ2 and h5 diameter tolerance; D10 permits a configured 35 mm length</x:v>
+      </x:c>
+      <x:c r="D20" s="212" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="E20" s="211" t="str">
+        <x:v>https://us.misumi-ec.com/vona2/detail/110302634310/</x:v>
+      </x:c>
+      <x:c r="F20" s="211" t="str">
+        <x:v>h5 is dimensionally compatible as a tighter subset of h6; verify US checkout and end/length finish.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="213" t="str">
+        <x:v>Engineering reference</x:v>
+      </x:c>
+      <x:c r="B21" s="211" t="str">
+        <x:v>WDS ISO shaft tolerance table</x:v>
+      </x:c>
+      <x:c r="C21" s="211" t="str">
+        <x:v>At nominal 10 mm: h6 is 9.991–10.000 mm while m6 is above nominal</x:v>
+      </x:c>
+      <x:c r="D21" s="212" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="E21" s="211" t="str">
+        <x:v>https://www.wdscomponents.com/en-gb/tolerances-for-holes-and-shafts</x:v>
+      </x:c>
+      <x:c r="F21" s="211" t="str">
+        <x:v>This is why a generic DIN 6325 m6 dowel is not an acceptable silent substitute.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="213" t="str">
+        <x:v>Current stock</x:v>
+      </x:c>
+      <x:c r="B22" s="211" t="str">
+        <x:v>DigiKey WAGO 221-413</x:v>
+      </x:c>
+      <x:c r="C22" s="211" t="str">
+        <x:v>Three-conductor lever connector, DigiKey 2946-221-413-ND</x:v>
+      </x:c>
+      <x:c r="D22" s="212" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="E22" s="211" t="str">
+        <x:v>https://www.digikey.com/en/products/detail/wago-corporation/221-413/13549610</x:v>
+      </x:c>
+      <x:c r="F22" s="211" t="str">
+        <x:v>Ordered 2026-08-31; actual checkout total was not provided.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>
@@ -4954,6 +5338,23 @@
         <x:v>Custom fallback</x:v>
       </x:c>
     </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="213" t="str">
+        <x:v>Ordered / in transit</x:v>
+      </x:c>
+      <x:c r="B42" s="213" t="str">
+        <x:v>WAGO 221-413 lever connector</x:v>
+      </x:c>
+      <x:c r="C42" s="213" t="str">
+        <x:v>DigiKey</x:v>
+      </x:c>
+      <x:c r="D42" s="213" t="str">
+        <x:v>https://www.digikey.com/en/products/detail/wago-corporation/221-413/13549610</x:v>
+      </x:c>
+      <x:c r="E42" s="213" t="str">
+        <x:v>Status &amp; Gaps ordered row 8</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:E1"/>
@@ -4961,4 +5362,543 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="11.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="13.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="21.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17.219999313354492" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="30.559999465942383" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="33.33000183105469" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="17.219999313354492" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="28.889999389648438" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="25.559999465942383" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28.5" customHeight="1">
+      <x:c r="A1" s="236" t="str">
+        <x:v>Mode A status — ordered inventory and remaining single-leg gaps</x:v>
+      </x:c>
+      <x:c r="B1" s="236"/>
+      <x:c r="C1" s="236"/>
+      <x:c r="D1" s="236"/>
+      <x:c r="E1" s="236"/>
+      <x:c r="F1" s="236"/>
+      <x:c r="G1" s="236"/>
+      <x:c r="H1" s="236"/>
+      <x:c r="I1" s="236"/>
+    </x:row>
+    <x:row r="2" ht="21" customHeight="1">
+      <x:c r="A2" s="237" t="str">
+        <x:v>Updated 2026-08-31 • ordered/in transit is deliberately separate from owned • exact-fit hardware is not silently substituted</x:v>
+      </x:c>
+      <x:c r="B2" s="237"/>
+      <x:c r="C2" s="237"/>
+      <x:c r="D2" s="237"/>
+      <x:c r="E2" s="237"/>
+      <x:c r="F2" s="237"/>
+      <x:c r="G2" s="237"/>
+      <x:c r="H2" s="237"/>
+      <x:c r="I2" s="237"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="238"/>
+      <x:c r="B3" s="238"/>
+      <x:c r="C3" s="238"/>
+      <x:c r="D3" s="238"/>
+      <x:c r="E3" s="238"/>
+      <x:c r="F3" s="238"/>
+      <x:c r="G3" s="238"/>
+      <x:c r="H3" s="238"/>
+      <x:c r="I3" s="238"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="239" t="str">
+        <x:v>ORDERED / IN TRANSIT — DIGIKEY ORDER</x:v>
+      </x:c>
+      <x:c r="B4" s="239"/>
+      <x:c r="C4" s="239"/>
+      <x:c r="D4" s="239"/>
+      <x:c r="E4" s="239"/>
+      <x:c r="F4" s="239"/>
+      <x:c r="G4" s="239"/>
+      <x:c r="H4" s="239"/>
+      <x:c r="I4" s="239"/>
+    </x:row>
+    <x:row r="5" ht="22.5" customHeight="1">
+      <x:c r="A5" s="240" t="str">
+        <x:v>Order date</x:v>
+      </x:c>
+      <x:c r="B5" s="240" t="str">
+        <x:v>State</x:v>
+      </x:c>
+      <x:c r="C5" s="240" t="str">
+        <x:v>Supplier</x:v>
+      </x:c>
+      <x:c r="D5" s="240" t="str">
+        <x:v>Category</x:v>
+      </x:c>
+      <x:c r="E5" s="240" t="str">
+        <x:v>Item</x:v>
+      </x:c>
+      <x:c r="F5" s="240" t="str">
+        <x:v>DigiKey SKU</x:v>
+      </x:c>
+      <x:c r="G5" s="240" t="str">
+        <x:v>Qty</x:v>
+      </x:c>
+      <x:c r="H5" s="240" t="str">
+        <x:v>Intended use</x:v>
+      </x:c>
+      <x:c r="I5" s="240" t="str">
+        <x:v>Receive &amp; verify</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="54" customHeight="1">
+      <x:c r="A6" s="241" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="B6" s="242" t="str">
+        <x:v>Ordered / in transit</x:v>
+      </x:c>
+      <x:c r="C6" s="242" t="str">
+        <x:v>DigiKey</x:v>
+      </x:c>
+      <x:c r="D6" s="242" t="str">
+        <x:v>CAN</x:v>
+      </x:c>
+      <x:c r="E6" s="242" t="str">
+        <x:v>Adafruit CAN Pal 5708</x:v>
+      </x:c>
+      <x:c r="F6" s="242" t="str">
+        <x:v>1528-5708-ND</x:v>
+      </x:c>
+      <x:c r="G6" s="242" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H6" s="242" t="str">
+        <x:v>One 3.3 V transceiver per Teensy CAN bus</x:v>
+      </x:c>
+      <x:c r="I6" s="242" t="str">
+        <x:v>With each board unpowered, enable termination and measure CANH–CANL ≈120 Ω.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="54" customHeight="1">
+      <x:c r="A7" s="241" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="B7" s="242" t="str">
+        <x:v>Ordered / in transit</x:v>
+      </x:c>
+      <x:c r="C7" s="242" t="str">
+        <x:v>DigiKey</x:v>
+      </x:c>
+      <x:c r="D7" s="242" t="str">
+        <x:v>Encoder</x:v>
+      </x:c>
+      <x:c r="E7" s="242" t="str">
+        <x:v>AS5048A adapter board kit</x:v>
+      </x:c>
+      <x:c r="F7" s="242" t="str">
+        <x:v>4991-AS5048AADAPTERBOARD-ND</x:v>
+      </x:c>
+      <x:c r="G7" s="242" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H7" s="242" t="str">
+        <x:v>Direct-SPI knee encoder</x:v>
+      </x:c>
+      <x:c r="I7" s="242" t="str">
+        <x:v>Confirm the loose AS5000-MD6H-2 diametric magnet is physically in the bag.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="54" customHeight="1">
+      <x:c r="A8" s="241" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="B8" s="242" t="str">
+        <x:v>Ordered / in transit</x:v>
+      </x:c>
+      <x:c r="C8" s="242" t="str">
+        <x:v>DigiKey</x:v>
+      </x:c>
+      <x:c r="D8" s="242" t="str">
+        <x:v>Encoder</x:v>
+      </x:c>
+      <x:c r="E8" s="242" t="str">
+        <x:v>1×8 male header</x:v>
+      </x:c>
+      <x:c r="F8" s="242" t="str">
+        <x:v>609-78511-108HLF-ND</x:v>
+      </x:c>
+      <x:c r="G8" s="242" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H8" s="242" t="str">
+        <x:v>Populate the adapter board's unpopulated P1</x:v>
+      </x:c>
+      <x:c r="I8" s="242" t="str">
+        <x:v>Dry-fit orientation before soldering; inspect every joint after soldering.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="54" customHeight="1">
+      <x:c r="A9" s="241" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="B9" s="242" t="str">
+        <x:v>Ordered / in transit</x:v>
+      </x:c>
+      <x:c r="C9" s="242" t="str">
+        <x:v>DigiKey</x:v>
+      </x:c>
+      <x:c r="D9" s="242" t="str">
+        <x:v>Power wiring</x:v>
+      </x:c>
+      <x:c r="E9" s="242" t="str">
+        <x:v>WAGO 221-413 three-conductor lever connector</x:v>
+      </x:c>
+      <x:c r="F9" s="242" t="str">
+        <x:v>2946-221-413-ND</x:v>
+      </x:c>
+      <x:c r="G9" s="242" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H9" s="242" t="str">
+        <x:v>Temporary bench power distribution; accepts the planned 18 AWG wire</x:v>
+      </x:c>
+      <x:c r="I9" s="242" t="str">
+        <x:v>Verify genuine WAGO marking, lever action and full conductor insertion; tug-test each wire.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="36" customHeight="1">
+      <x:c r="A10" s="238"/>
+      <x:c r="B10" s="238"/>
+      <x:c r="C10" s="238"/>
+      <x:c r="D10" s="238"/>
+      <x:c r="E10" s="238"/>
+      <x:c r="F10" s="238"/>
+      <x:c r="G10" s="238"/>
+      <x:c r="H10" s="238"/>
+      <x:c r="I10" s="238"/>
+    </x:row>
+    <x:row r="11" ht="36" customHeight="1">
+      <x:c r="A11" s="239" t="str">
+        <x:v>INITIAL SINGLE-LEG TEST READINESS</x:v>
+      </x:c>
+      <x:c r="B11" s="239"/>
+      <x:c r="C11" s="239"/>
+      <x:c r="D11" s="239"/>
+      <x:c r="E11" s="239"/>
+      <x:c r="F11" s="239"/>
+      <x:c r="G11" s="239"/>
+      <x:c r="H11" s="239"/>
+      <x:c r="I11" s="239"/>
+    </x:row>
+    <x:row r="12" ht="27" customHeight="1">
+      <x:c r="A12" s="240" t="str">
+        <x:v>Phase / gate</x:v>
+      </x:c>
+      <x:c r="B12" s="240" t="str">
+        <x:v>State</x:v>
+      </x:c>
+      <x:c r="C12" s="240" t="str">
+        <x:v>Item</x:v>
+      </x:c>
+      <x:c r="D12" s="240" t="str">
+        <x:v>Where tracked</x:v>
+      </x:c>
+      <x:c r="E12" s="240" t="str">
+        <x:v>Next action</x:v>
+      </x:c>
+      <x:c r="F12" s="240" t="str">
+        <x:v>Why / compatibility</x:v>
+      </x:c>
+      <x:c r="G12" s="240" t="str">
+        <x:v>Buy timing</x:v>
+      </x:c>
+      <x:c r="H12" s="240" t="str">
+        <x:v>Lowest-cost path</x:v>
+      </x:c>
+      <x:c r="I12" s="240" t="str">
+        <x:v>Source / evidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="57" customHeight="1">
+      <x:c r="A13" s="243" t="str">
+        <x:v>ABS fit</x:v>
+      </x:c>
+      <x:c r="B13" s="244" t="str">
+        <x:v>BLOCKED</x:v>
+      </x:c>
+      <x:c r="C13" s="243" t="str">
+        <x:v>Ø10 h6 × 35 mm hardened/ground knee axle</x:v>
+      </x:c>
+      <x:c r="D13" s="243" t="str">
+        <x:v>RFQ &amp; Holds row 6</x:v>
+      </x:c>
+      <x:c r="E13" s="243" t="str">
+        <x:v>Ask WDS to certify 9.991–10.000 mm; otherwise verify MISUMI PSFU10-35 h5.</x:v>
+      </x:c>
+      <x:c r="F13" s="243" t="str">
+        <x:v>This pin is the printed-bore fit gauge and the AS5048A angular datum. A common m6 dowel can be oversize.</x:v>
+      </x:c>
+      <x:c r="G13" s="243" t="str">
+        <x:v>Now</x:v>
+      </x:c>
+      <x:c r="H13" s="243" t="str">
+        <x:v>WDS is $1.31 if certified; do not spend on an unverified near-match.</x:v>
+      </x:c>
+      <x:c r="I13" s="243" t="str">
+        <x:v>WDS 662-20635 / MISUMI PSFU10-35</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="57" customHeight="1">
+      <x:c r="A14" s="243" t="str">
+        <x:v>ABS fit</x:v>
+      </x:c>
+      <x:c r="B14" s="245" t="str">
+        <x:v>IN PROGRESS</x:v>
+      </x:c>
+      <x:c r="C14" s="243" t="str">
+        <x:v>6800 bearing-seat ladder</x:v>
+      </x:c>
+      <x:c r="D14" s="243" t="str">
+        <x:v>README / first_article_stl</x:v>
+      </x:c>
+      <x:c r="E14" s="243" t="str">
+        <x:v>Test the owned bearing from Ø19.05 upward and stop at the first firm thumb fit with no rock.</x:v>
+      </x:c>
+      <x:c r="F14" s="243" t="str">
+        <x:v>The nominal Ø19.00 coupon failed; forcing the bearing risks scarring it or splitting ABS.</x:v>
+      </x:c>
+      <x:c r="G14" s="243" t="str">
+        <x:v>Before full link print</x:v>
+      </x:c>
+      <x:c r="H14" s="243" t="str">
+        <x:v>$0 — use the owned bearing and existing ladder STL.</x:v>
+      </x:c>
+      <x:c r="I14" s="243" t="str">
+        <x:v>README.md lines 38–46</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="57" customHeight="1">
+      <x:c r="A15" s="243" t="str">
+        <x:v>Bench electronics</x:v>
+      </x:c>
+      <x:c r="B15" s="245" t="str">
+        <x:v>PARTLY ORDERED</x:v>
+      </x:c>
+      <x:c r="C15" s="243" t="str">
+        <x:v>CAN + encoder ordered; bench PSU and microSD remain open</x:v>
+      </x:c>
+      <x:c r="D15" s="243" t="str">
+        <x:v>Order Now rows 5–9</x:v>
+      </x:c>
+      <x:c r="E15" s="243" t="str">
+        <x:v>Receive/verify DigiKey parts; buy/borrow current-limited PSU and obtain tested microSD before powered work.</x:v>
+      </x:c>
+      <x:c r="F15" s="243" t="str">
+        <x:v>CAN/encoder parts are compatible with the Teensy 3.3 V path; the actuator stage still needs a 20 V current-limited source.</x:v>
+      </x:c>
+      <x:c r="G15" s="243" t="str">
+        <x:v>Before steps 1–2</x:v>
+      </x:c>
+      <x:c r="H15" s="243" t="str">
+        <x:v>Use existing USB power for logic-only checks; do not power an actuator without a current-limited supply.</x:v>
+      </x:c>
+      <x:c r="I15" s="243" t="str">
+        <x:v>electronics/07_bom.md Wave 0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="57" customHeight="1">
+      <x:c r="A16" s="243" t="str">
+        <x:v>Mechanical assembly</x:v>
+      </x:c>
+      <x:c r="B16" s="246" t="str">
+        <x:v>OPEN / RFQ</x:v>
+      </x:c>
+      <x:c r="C16" s="243" t="str">
+        <x:v>Main spring, Ø6 h6 stop pin, Ø5 h6 guide shaft, Ø19/Ø13.6 preload shims</x:v>
+      </x:c>
+      <x:c r="D16" s="243" t="str">
+        <x:v>RFQ &amp; Holds rows 5, 7–9</x:v>
+      </x:c>
+      <x:c r="E16" s="243" t="str">
+        <x:v>Request exact drawings/certificates; do not substitute rounded catalog sizes.</x:v>
+      </x:c>
+      <x:c r="F16" s="243" t="str">
+        <x:v>These parts set spring rate, −8° stop engagement, cartridge alignment and preload.</x:v>
+      </x:c>
+      <x:c r="G16" s="243" t="str">
+        <x:v>Now for Mode A through step 6</x:v>
+      </x:c>
+      <x:c r="H16" s="243" t="str">
+        <x:v>Bundle RFQs where possible; A228 music-wire spring is acceptable for the early prototype.</x:v>
+      </x:c>
+      <x:c r="I16" s="243" t="str">
+        <x:v>beni_single_leg_rig_design_record.md §9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="57" customHeight="1">
+      <x:c r="A17" s="243" t="str">
+        <x:v>Mechanical assembly</x:v>
+      </x:c>
+      <x:c r="B17" s="244" t="str">
+        <x:v>DESIGN HOLD</x:v>
+      </x:c>
+      <x:c r="C17" s="243" t="str">
+        <x:v>2 × Ø4 × 32 clevis pins plus retention</x:v>
+      </x:c>
+      <x:c r="D17" s="243" t="str">
+        <x:v>RFQ &amp; Holds row 10</x:v>
+      </x:c>
+      <x:c r="E17" s="243" t="str">
+        <x:v>Close the retention scheme in Fusion before buying pin/ring/cotter hardware.</x:v>
+      </x:c>
+      <x:c r="F17" s="243" t="str">
+        <x:v>The active body has no verified E-clip groove or cross-hole; the cartridge must not shed a pin.</x:v>
+      </x:c>
+      <x:c r="G17" s="243" t="str">
+        <x:v>Before installing spring cartridge</x:v>
+      </x:c>
+      <x:c r="H17" s="243" t="str">
+        <x:v>Do not buy twice; wait for the exact retention geometry.</x:v>
+      </x:c>
+      <x:c r="I17" s="243" t="str">
+        <x:v>Fusion hold recorded in workbook</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="57" customHeight="1">
+      <x:c r="A18" s="243" t="str">
+        <x:v>Knee bearing stack</x:v>
+      </x:c>
+      <x:c r="B18" s="246" t="str">
+        <x:v>CHECK WORKSHOP</x:v>
+      </x:c>
+      <x:c r="C18" s="243" t="str">
+        <x:v>2 × PTFE/POM thrust washers, Ø22/Ø16.5 × 0.5, as required</x:v>
+      </x:c>
+      <x:c r="D18" s="243" t="str">
+        <x:v>Not previously in procurement tracker</x:v>
+      </x:c>
+      <x:c r="E18" s="243" t="str">
+        <x:v>Dry-fit the exact pin/link stack; buy only if axial fit calls for them, and keep the stated dimensions.</x:v>
+      </x:c>
+      <x:c r="F18" s="243" t="str">
+        <x:v>The assembly BOM places one washer on each side of the distal link; they are explicitly 'as required.'</x:v>
+      </x:c>
+      <x:c r="G18" s="243" t="str">
+        <x:v>Before final knee assembly</x:v>
+      </x:c>
+      <x:c r="H18" s="243" t="str">
+        <x:v>Inventory first; do not buy a 50-piece specialty pack unless the dry fit proves the need.</x:v>
+      </x:c>
+      <x:c r="I18" s="243" t="str">
+        <x:v>beni_prototype1_bom_and_assembly.md A1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="57" customHeight="1">
+      <x:c r="A19" s="243" t="str">
+        <x:v>Assembly consumables</x:v>
+      </x:c>
+      <x:c r="B19" s="246" t="str">
+        <x:v>CHECK WORKSHOP</x:v>
+      </x:c>
+      <x:c r="C19" s="243" t="str">
+        <x:v>M3 set screw, retaining compound and magnet adhesive</x:v>
+      </x:c>
+      <x:c r="D19" s="243" t="str">
+        <x:v>Not previously in procurement tracker</x:v>
+      </x:c>
+      <x:c r="E19" s="243" t="str">
+        <x:v>Confirm compatible sizes/chemistry after the printed collar and carrier are dry-fitted.</x:v>
+      </x:c>
+      <x:c r="F19" s="243" t="str">
+        <x:v>The active knee retention uses an M3 set screw plus retaining compound; the diametric magnet must be bonded securely.</x:v>
+      </x:c>
+      <x:c r="G19" s="243" t="str">
+        <x:v>Before final knee assembly</x:v>
+      </x:c>
+      <x:c r="H19" s="243" t="str">
+        <x:v>Use existing workshop stock if suitable; these are tiny quantities.</x:v>
+      </x:c>
+      <x:c r="I19" s="243" t="str">
+        <x:v>beni_single_leg_rig_design_record.md §4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="57" customHeight="1">
+      <x:c r="A20" s="243" t="str">
+        <x:v>Mode A instruments</x:v>
+      </x:c>
+      <x:c r="B20" s="246" t="str">
+        <x:v>CHECK / BORROW</x:v>
+      </x:c>
+      <x:c r="C20" s="243" t="str">
+        <x:v>5 kg scale + known masses; dial indicator; DMM; 4-wire milliohm meter; 2-channel scope/logic analyzer</x:v>
+      </x:c>
+      <x:c r="D20" s="243" t="str">
+        <x:v>Conditional plus test brief steps 2–4</x:v>
+      </x:c>
+      <x:c r="E20" s="243" t="str">
+        <x:v>Inventory or borrow first. A normal DMM does not replace the milliohm measurement; latency needs two observable timing channels.</x:v>
+      </x:c>
+      <x:c r="F20" s="243" t="str">
+        <x:v>These gate torque, phase resistance, magnet-carrier TIR and &lt;8 ms loop latency.</x:v>
+      </x:c>
+      <x:c r="G20" s="243" t="str">
+        <x:v>Before steps 2–4</x:v>
+      </x:c>
+      <x:c r="H20" s="243" t="str">
+        <x:v>Borrowing is the cheapest high-confidence option; buy only what cannot be borrowed.</x:v>
+      </x:c>
+      <x:c r="I20" s="243" t="str">
+        <x:v>fusion_brief_single_leg_rig.md §6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="57" customHeight="1">
+      <x:c r="A21" s="243" t="str">
+        <x:v>Structural release</x:v>
+      </x:c>
+      <x:c r="B21" s="247" t="str">
+        <x:v>AFTER ABS FIT</x:v>
+      </x:c>
+      <x:c r="C21" s="243" t="str">
+        <x:v>PA6-CF and hardened 0.6 mm hotend</x:v>
+      </x:c>
+      <x:c r="D21" s="243" t="str">
+        <x:v>Conditional rows 12–13</x:v>
+      </x:c>
+      <x:c r="E21" s="243" t="str">
+        <x:v>Buy only if not already owned, after ABS geometry passes; re-run critical PA-CF fit coupons.</x:v>
+      </x:c>
+      <x:c r="F21" s="243" t="str">
+        <x:v>ABS is for unloaded fit/assembly only. Torque and spring loading require the structural material release.</x:v>
+      </x:c>
+      <x:c r="G21" s="243" t="str">
+        <x:v>After ABS fit; before torque/spring loads</x:v>
+      </x:c>
+      <x:c r="H21" s="243" t="str">
+        <x:v>Do not consume the PA-CF spool during fit iteration.</x:v>
+      </x:c>
+      <x:c r="I21" s="243" t="str">
+        <x:v>CLAUDE.md hard rule 7</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:I1"/>
+    <x:mergeCell ref="A2:I2"/>
+    <x:mergeCell ref="A4:I4"/>
+    <x:mergeCell ref="A11:I11"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="2">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0079a13c4fcd4d70"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R405c2671a7314188"/>
+  </x:tableParts>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record proximal bearing fit and ABS build scope
</commit_message>
<xml_diff>
--- a/procurement/mode_a_procurement_bom_2026-08-21.xlsx
+++ b/procurement/mode_a_procurement_bom_2026-08-21.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R6104ca8232a44355"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order Now" sheetId="2" r:id="R2c6a12c4dcf64474"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conditional" sheetId="3" r:id="R920cfae8e15e42f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ &amp; Holds" sheetId="4" r:id="Rc338f2202a2a4427"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplier Carts" sheetId="5" r:id="Rd0c8fa95d680436f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owned &amp; Printed" sheetId="6" r:id="R917f6ba2bbd14e92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" r:id="R5cefc1164b6e4fb7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order Links" sheetId="8" r:id="Rc60e9ae50ab74bdc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status &amp; Gaps" sheetId="9" r:id="R06172480efc546b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Rc272015197034a95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order Now" sheetId="2" r:id="R0bbd23ccf2b24d1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conditional" sheetId="3" r:id="Rac4c091a23d34bb8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ &amp; Holds" sheetId="4" r:id="R2534a57dd14544ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplier Carts" sheetId="5" r:id="R6b1daee730a846f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owned &amp; Printed" sheetId="6" r:id="R47916313bedb46e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" r:id="R9b6ff4c2aae44a11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order Links" sheetId="8" r:id="R7eaf3f4faae94f47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status &amp; Gaps" sheetId="9" r:id="R5e722ed5af2248fb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -611,7 +611,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="248">
+  <x:cellXfs count="249">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1206,6 +1206,9 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="53" fillId="11" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1468,7 +1471,7 @@
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
       <x:c r="A2" s="146" t="str">
-        <x:v>Los Altos, California • procurement status updated 2026-08-31 • ABS fit campaign first • all structural PA-CF and Fusion release gates preserved</x:v>
+        <x:v>Los Altos, California • procurement status updated 2026-09-02 • complete ABS single-leg integration first • PA-CF deferred to the later two-leg structural build</x:v>
       </x:c>
       <x:c r="B2" s="146"/>
       <x:c r="C2" s="146"/>
@@ -1513,12 +1516,12 @@
       <x:c r="C5" s="147"/>
       <x:c r="D5" s="156" t="n">
         <x:f>SUMIF(Conditional!$A$5:$A$13,"Now if missing",Conditional!$H$5:$H$13)</x:f>
-        <x:v>72.54</x:v>
+        <x:v>62.75000000000001</x:v>
       </x:c>
       <x:c r="E5" s="157"/>
       <x:c r="F5" s="147"/>
       <x:c r="G5" s="158" t="str">
-        <x:v>5 RFQ + 1 CAD HOLD</x:v>
+        <x:v>4 RFQ + VERIFY + HOLD</x:v>
       </x:c>
       <x:c r="H5" s="159"/>
     </x:row>
@@ -1570,15 +1573,15 @@
       <x:c r="G9" s="147"/>
       <x:c r="H9" s="147"/>
     </x:row>
-    <x:row r="10" ht="42" customHeight="1">
+    <x:row r="10" ht="68" customHeight="1">
       <x:c r="A10" s="167" t="str">
         <x:v>2</x:v>
       </x:c>
       <x:c r="B10" s="168" t="str">
-        <x:v>Inventory the conditional lines before checkout</x:v>
+        <x:v>Inventory active-phase essentials</x:v>
       </x:c>
       <x:c r="C10" s="169" t="str">
-        <x:v>In particular: 16–18 AWG power wire, DMM, dial indicator, 5 kg scale, metric hex keys, TPU, hardened 0.6 hotend, and the physical AS5048 magnet.</x:v>
+        <x:v>16–18 AWG stranded copper wire, polarized power connectors, ferrules, heat-shrink, a DMM, dial indicator, access to a 4-wire milliohm meter and 2-channel scope/logic analyzer, hex keys, a microSD card, TPU 95A, and general assembly hardware. Defer the 5 kg scale, force/torque metrology, and PA-CF hotend/nozzle release until the later two-leg build.</x:v>
       </x:c>
       <x:c r="D10" s="147"/>
       <x:c r="E10" s="147"/>
@@ -1623,10 +1626,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B13" s="168" t="str">
-        <x:v>After ABS fit passes</x:v>
+        <x:v>After the complete ABS single-leg integration article</x:v>
       </x:c>
       <x:c r="C13" s="169" t="str">
-        <x:v>Buy PA6-CF and the hardened 0.6 hotend only if not already owned; reprint structural load paths before spring, torque or proof loading.</x:v>
+        <x:v>Keep PA6-CF and the hardened 0.6 hotend deferred until the two-leg structural build. The ABS leg may run self-weight-only, wheel-clear, current-limited motor/electronics checks; no spring characterization, ground traction, stall/proof torque or drops through ABS.</x:v>
       </x:c>
       <x:c r="D13" s="147"/>
       <x:c r="E13" s="147"/>
@@ -1694,7 +1697,7 @@
     </x:row>
     <x:row r="19" ht="31" customHeight="1">
       <x:c r="A19" s="171" t="str">
-        <x:v>• ABS is for fit/assembly. Any torque, spring, human-adjacent or proof-loading campaign waits for structural PA-CF parts and the recorded release gates.</x:v>
+        <x:v>• The active build remains ABS through the complete single-leg integration article. Current-limited, wheel-clear, self-weight-only motor/electronics checks are allowed; spring characterization, ground traction, stall/proof torque, drops and other structural loads wait for the two-leg PA-CF build.</x:v>
       </x:c>
       <x:c r="B19" s="171"/>
       <x:c r="C19" s="171"/>
@@ -1861,7 +1864,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="146" t="str">
-        <x:v>One ABS fit/assembly leg plus the first safe powered bench campaign. Status updated 2026-08-31; tax and shipping are excluded. The subtotal includes only still-open lines.</x:v>
+        <x:v>One complete ABS single-leg integration article plus wheel-clear/current-limited motor and electronics checks. Status updated 2026-09-02; tax and shipping are excluded. The subtotal includes only still-open lines.</x:v>
       </x:c>
       <x:c r="B2" s="146"/>
       <x:c r="C2" s="146"/>
@@ -2876,7 +2879,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="146" t="str">
-        <x:v>These are real build needs, but buying duplicates would waste money. The trigger column says exactly when to add each line. “Later” material lines remain outside the ABS fit campaign.</x:v>
+        <x:v>Buy these only when the trigger is reached. PA-CF/PA-GF structural-print items remain outside the ABS single-leg integration phase.</x:v>
       </x:c>
       <x:c r="B2" s="146"/>
       <x:c r="C2" s="146"/>
@@ -3100,7 +3103,7 @@
     </x:row>
     <x:row r="9" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A9" s="181" t="str">
-        <x:v>Now if missing</x:v>
+        <x:v>Two-leg structural build</x:v>
       </x:c>
       <x:c r="B9" s="176" t="str">
         <x:v>Metrology</x:v>
@@ -3112,7 +3115,7 @@
         <x:v>Gram display, tare function, ≥5 kg capacity</x:v>
       </x:c>
       <x:c r="E9" s="176" t="str">
-        <x:v>Buy or borrow before the force/torque characterization campaign.</x:v>
+        <x:v>Buy or borrow before the deferred force/torque and spring-characterization campaign.</x:v>
       </x:c>
       <x:c r="F9" s="176" t="n">
         <x:v>1</x:v>
@@ -3134,7 +3137,7 @@
         <x:v>URL tab →</x:v>
       </x:c>
       <x:c r="L9" s="176" t="str">
-        <x:v>Use known water masses or verified household masses; no calipers are required for the current coupon-first fit process.</x:v>
+        <x:v>Not required for wiring, latency, CAN soak or wheel-clear/current-limited commissioning. Use known water masses or verified masses later.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -3217,7 +3220,7 @@
     </x:row>
     <x:row r="12" ht="32.400001525878906" hidden="0" customHeight="1">
       <x:c r="A12" s="183" t="str">
-        <x:v>After ABS fit</x:v>
+        <x:v>Two-leg structural build</x:v>
       </x:c>
       <x:c r="B12" s="176" t="str">
         <x:v>Material</x:v>
@@ -3229,7 +3232,7 @@
         <x:v>Bambu Lab PA6-CF, initial 1 kg spool</x:v>
       </x:c>
       <x:c r="E12" s="176" t="str">
-        <x:v>Buy after ABS geometry/fit is accepted and before torque, spring or proof loading.</x:v>
+        <x:v>Buy immediately before the two-leg structural prints, after the complete ABS single-leg integration article is accepted.</x:v>
       </x:c>
       <x:c r="F12" s="176" t="n">
         <x:v>1</x:v>
@@ -3251,12 +3254,12 @@
         <x:v>URL tab →</x:v>
       </x:c>
       <x:c r="L12" s="176" t="str">
-        <x:v>One initial spool is a purchasing unit, not a claim that the full structural campaign consumes exactly 1 kg; confirm slicer mass before reordering.</x:v>
+        <x:v>Deferred by owner decision 2026-09-02 until the two-leg structural build; do not buy for the ABS single-leg integration article.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A13" s="183" t="str">
-        <x:v>After ABS fit</x:v>
+        <x:v>Two-leg structural build</x:v>
       </x:c>
       <x:c r="B13" s="176" t="str">
         <x:v>Printer</x:v>
@@ -3268,7 +3271,7 @@
         <x:v>Bambu hotend for H2 Series, 0.6 mm hardened nozzle</x:v>
       </x:c>
       <x:c r="E13" s="176" t="str">
-        <x:v>Buy only if your H2S does not already have the hardened 0.6 mm hotend needed for filled PA6-CF.</x:v>
+        <x:v>Buy with PA6-CF only if the selected printer does not already have the required hardened 0.6 mm hotend.</x:v>
       </x:c>
       <x:c r="F13" s="176" t="n">
         <x:v>1</x:v>
@@ -3290,7 +3293,7 @@
         <x:v>URL tab →</x:v>
       </x:c>
       <x:c r="L13" s="176" t="str">
-        <x:v>Required by the project’s PA-CF printing setup, not by the ABS fit campaign.</x:v>
+        <x:v>Deferred with PA6-CF until the two-leg structural build; inventory first and buy only if missing then.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -3444,25 +3447,25 @@
     </x:row>
     <x:row r="6" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A6" s="198" t="str">
-        <x:v>RFQ / VERIFY — NO m6 SUBSTITUTE</x:v>
+        <x:v>ORDERED / VERIFY — NO m6 SUBSTITUTE</x:v>
       </x:c>
       <x:c r="B6" s="176" t="str">
         <x:v>Pins</x:v>
       </x:c>
       <x:c r="C6" s="176" t="str">
-        <x:v>Ø10 h6 × 35 hardened ground dowel</x:v>
+        <x:v>Owner-reported eBay candidate Ø10 × 35 knee pins</x:v>
       </x:c>
       <x:c r="D6" s="176" t="str">
         <x:v>10.000/−0.009 mm (ISO h6), 35 mm finished length, hardened and ground</x:v>
       </x:c>
-      <x:c r="E6" s="176" t="n">
-        <x:v>1</x:v>
+      <x:c r="E6" s="176" t="str">
+        <x:v>Believed 3; verify</x:v>
       </x:c>
       <x:c r="F6" s="176" t="str">
-        <x:v>WDS 662-20635 is catalogued as 10 × 35 mm hardened/ground at $1.31, but its page omits diameter tolerance. Ask WDS for written 9.991–10.000 mm confirmation; order only if confirmed.</x:v>
+        <x:v>Wait for the package (owner estimate: roughly two weeks or later); record the listing/item ID, count the pins, and verify 35 mm length plus 9.991–10.000 mm h6 or acceptable h5 evidence before release.</x:v>
       </x:c>
       <x:c r="G6" s="178" t="str">
-        <x:v>WDS Components</x:v>
+        <x:v>eBay — owner order; listing not recorded</x:v>
       </x:c>
       <x:c r="H6" s="178" t="str">
         <x:v>MISUMI PSFU10-35: hardened SUJ2, h5 (a tighter subset of h6). Verify US availability, finished-length tolerance and usable end face before ordering.</x:v>
@@ -3471,7 +3474,7 @@
         <x:v>Common DIN 6325 dowels are usually m6 (positive tolerance) and can interfere with a nominal 10 mm bearing bore. A shoulder bolt is too loose for the angular datum.</x:v>
       </x:c>
       <x:c r="J6" s="176" t="str">
-        <x:v>Supplier certificate/drawing explicitly stating h6, or the verified MISUMI h5 drawing plus acceptable end and length finish.</x:v>
+        <x:v>Recorded listing/package count and specification, plus h6/h5 evidence and successful hand fit through both 6800 bearings and the vertical Ø10 coupon.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="21.600000381469727" hidden="0" customHeight="1">
@@ -4115,7 +4118,7 @@
         <x:v>Owner update</x:v>
       </x:c>
       <x:c r="F11" s="176" t="str">
-        <x:v>Confirm installed nozzle/hotend before PA-CF release.</x:v>
+        <x:v>Confirm the installed nozzle/hotend and dry-box path before the later two-leg PA-CF build.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
@@ -4126,16 +4129,16 @@
         <x:v>Material</x:v>
       </x:c>
       <x:c r="C12" s="176" t="str">
-        <x:v>ABS</x:v>
+        <x:v>Active ABS single-leg integration material</x:v>
       </x:c>
       <x:c r="D12" s="176" t="str">
-        <x:v>Owner has a large supply</x:v>
+        <x:v>In use</x:v>
       </x:c>
       <x:c r="E12" s="176" t="str">
-        <x:v>Owner directive / CLAUDE.md rule 7</x:v>
+        <x:v>Low-load fit, assembly, wiring, controls integration, and wheel-clear/current-limited slow motor commands under self-weight only</x:v>
       </x:c>
       <x:c r="F12" s="176" t="str">
-        <x:v>Use for first fit and assembly only.</x:v>
+        <x:v>Do not use ABS for torque-arm, main-spring preload/characterization, ground-traction, stall/proof, drop, or human-adjacent tests.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -4166,16 +4169,16 @@
         <x:v>Mode A rig</x:v>
       </x:c>
       <x:c r="C14" s="176" t="str">
-        <x:v>Stand, torque arm, floor plate, Cable Post A, stop/bumper/collar/magnet carrier and leg parts</x:v>
+        <x:v>ABS first-article proximal link printed; complete the remaining single-leg fit and integration work</x:v>
       </x:c>
       <x:c r="D14" s="176" t="str">
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="E14" s="176" t="str">
-        <x:v>Current owner update</x:v>
+        <x:v>Single-leg geometry and unloaded controls integration only</x:v>
       </x:c>
       <x:c r="F14" s="176" t="str">
-        <x:v>Dry-fit and log every interference before structural reprint.</x:v>
+        <x:v>The current Ø19.10 proximal link is retained. Do not apply structural or spring loads to the ABS assembly.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="32.400001525878906" hidden="0" customHeight="1">
@@ -4195,7 +4198,7 @@
         <x:v>README.md / owner update</x:v>
       </x:c>
       <x:c r="F15" s="206" t="str">
-        <x:v>Use one real bearing for the indexed ABS bore-ladder test; do not force it into the failed Ø19.00 coupon.</x:v>
+        <x:v>Full-depth Ø19.10 ABS link accepts both bearings but is slightly tight; use Ø19.15 for future ABS proximal-link prints.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -5136,7 +5139,7 @@
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
       <x:c r="A30" s="176" t="str">
-        <x:v>Now if missing</x:v>
+        <x:v>Two-leg structural build</x:v>
       </x:c>
       <x:c r="B30" s="176" t="str">
         <x:v>5 kg / 11 lb digital kitchen scale</x:v>
@@ -5187,7 +5190,7 @@
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
       <x:c r="A33" s="176" t="str">
-        <x:v>After ABS fit</x:v>
+        <x:v>Two-leg structural build</x:v>
       </x:c>
       <x:c r="B33" s="176" t="str">
         <x:v>PA6-CF</x:v>
@@ -5204,7 +5207,7 @@
     </x:row>
     <x:row r="34" ht="15" hidden="0" customHeight="1">
       <x:c r="A34" s="176" t="str">
-        <x:v>After ABS fit</x:v>
+        <x:v>Two-leg structural build</x:v>
       </x:c>
       <x:c r="B34" s="176" t="str">
         <x:v>0.6 mm hardened hotend</x:v>
@@ -5238,19 +5241,19 @@
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
       <x:c r="A36" s="176" t="str">
-        <x:v>RFQ / verify</x:v>
+        <x:v>Ordered / verify</x:v>
       </x:c>
       <x:c r="B36" s="176" t="str">
-        <x:v>Ø10 h6 × 35 hardened ground dowel</x:v>
+        <x:v>Candidate Ø10 × 35 knee pins (h6/h5 not yet evidenced)</x:v>
       </x:c>
       <x:c r="C36" s="176" t="str">
-        <x:v>WDS Components</x:v>
+        <x:v>eBay — owner order</x:v>
       </x:c>
       <x:c r="D36" s="192" t="str">
-        <x:v>https://www.wdscomponents.com/en-us/10mm-x-35mm-steel-precision-dowel-pin</x:v>
+        <x:v>Owner eBay listing URL / item ID not recorded</x:v>
       </x:c>
       <x:c r="E36" s="176" t="str">
-        <x:v>RFQ &amp; Holds row 6</x:v>
+        <x:v>RFQ &amp; Holds row 6; owner report 2026-09-02</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
@@ -5394,7 +5397,7 @@
     </x:row>
     <x:row r="2" ht="21" customHeight="1">
       <x:c r="A2" s="237" t="str">
-        <x:v>Updated 2026-08-31 • ordered/in transit is deliberately separate from owned • exact-fit hardware is not silently substituted</x:v>
+        <x:v>Updated 2026-09-02 • ordered/in transit is deliberately separate from owned • exact-fit hardware is not silently substituted</x:v>
       </x:c>
       <x:c r="B2" s="237"/>
       <x:c r="C2" s="237"/>
@@ -5574,16 +5577,34 @@
         <x:v>Verify genuine WAGO marking, lever action and full conductor insertion; tug-test each wire.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="36" customHeight="1">
-      <x:c r="A10" s="238"/>
-      <x:c r="B10" s="238"/>
-      <x:c r="C10" s="238"/>
-      <x:c r="D10" s="238"/>
-      <x:c r="E10" s="238"/>
-      <x:c r="F10" s="238"/>
-      <x:c r="G10" s="238"/>
-      <x:c r="H10" s="238"/>
-      <x:c r="I10" s="238"/>
+    <x:row r="10" ht="72" customHeight="1">
+      <x:c r="A10" s="248" t="str">
+        <x:v>2026-09-02</x:v>
+      </x:c>
+      <x:c r="B10" s="248" t="str">
+        <x:v>Ordered / in transit — verify</x:v>
+      </x:c>
+      <x:c r="C10" s="248" t="str">
+        <x:v>eBay — owner report</x:v>
+      </x:c>
+      <x:c r="D10" s="248" t="str">
+        <x:v>Pins</x:v>
+      </x:c>
+      <x:c r="E10" s="248" t="str">
+        <x:v>Candidate knee pins; believed set of 3</x:v>
+      </x:c>
+      <x:c r="F10" s="248" t="str">
+        <x:v>Listing / item ID not recorded</x:v>
+      </x:c>
+      <x:c r="G10" s="248" t="str">
+        <x:v>3? — verify</x:v>
+      </x:c>
+      <x:c r="H10" s="248" t="str">
+        <x:v>Candidate Ø10 h6/h5 × 35 mm knee axle and fit gate</x:v>
+      </x:c>
+      <x:c r="I10" s="248" t="str">
+        <x:v>On arrival, record the listing and count; verify Ø10 × 35, h6/h5 evidence, bearing hand fit and vertical coupon fit. ETA owner estimate: roughly two weeks or later.</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="36" customHeight="1">
       <x:c r="A11" s="239" t="str">
@@ -5632,28 +5653,28 @@
         <x:v>ABS fit</x:v>
       </x:c>
       <x:c r="B13" s="244" t="str">
-        <x:v>BLOCKED</x:v>
+        <x:v>ORDERED — VERIFY</x:v>
       </x:c>
       <x:c r="C13" s="243" t="str">
-        <x:v>Ø10 h6 × 35 mm hardened/ground knee axle</x:v>
+        <x:v>eBay candidate knee pins; believed set of 3</x:v>
       </x:c>
       <x:c r="D13" s="243" t="str">
-        <x:v>RFQ &amp; Holds row 6</x:v>
+        <x:v>RFQ &amp; Holds row 6 / owner report 2026-09-02</x:v>
       </x:c>
       <x:c r="E13" s="243" t="str">
-        <x:v>Ask WDS to certify 9.991–10.000 mm; otherwise verify MISUMI PSFU10-35 h5.</x:v>
+        <x:v>Wait for arrival; record listing and quantity, then verify Ø10 × 35 mm plus h6/h5 evidence, both bearing bores and the vertical fit coupon.</x:v>
       </x:c>
       <x:c r="F13" s="243" t="str">
-        <x:v>This pin is the printed-bore fit gauge and the AS5048A angular datum. A common m6 dowel can be oversize.</x:v>
+        <x:v>A common m6 dowel can be oversize. A printed ABS pin is only a supported hand-alignment placeholder and cannot clear this gate.</x:v>
       </x:c>
       <x:c r="G13" s="243" t="str">
-        <x:v>Now</x:v>
+        <x:v>ETA roughly 2026-09-16 or later — verify</x:v>
       </x:c>
       <x:c r="H13" s="243" t="str">
-        <x:v>WDS is $1.31 if certified; do not spend on an unverified near-match.</x:v>
+        <x:v>$0 additional now; use the eBay order if it proves compliant.</x:v>
       </x:c>
       <x:c r="I13" s="243" t="str">
-        <x:v>WDS 662-20635 / MISUMI PSFU10-35</x:v>
+        <x:v>Owner report only; seller listing and package evidence pending</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="57" customHeight="1">
@@ -5661,25 +5682,25 @@
         <x:v>ABS fit</x:v>
       </x:c>
       <x:c r="B14" s="245" t="str">
-        <x:v>IN PROGRESS</x:v>
+        <x:v>COMPLETE</x:v>
       </x:c>
       <x:c r="C14" s="243" t="str">
-        <x:v>6800 bearing-seat ladder</x:v>
+        <x:v>6800 bearing ladder + full-depth proximal link</x:v>
       </x:c>
       <x:c r="D14" s="243" t="str">
-        <x:v>README / first_article_stl</x:v>
+        <x:v>evidence/knee_fit/2026-09-02_proximal_link_full_depth</x:v>
       </x:c>
       <x:c r="E14" s="243" t="str">
-        <x:v>Test the owned bearing from Ø19.05 upward and stop at the first firm thumb fit with no rock.</x:v>
+        <x:v>Keep the existing Ø19.10 ABS link; use Ø19.15 as the preferred compensation for any future ABS proximal print.</x:v>
       </x:c>
       <x:c r="F14" s="243" t="str">
-        <x:v>The nominal Ø19.00 coupon failed; forcing the bearing risks scarring it or splitting ABS.</x:v>
+        <x:v>The full-depth Ø19.10 seats accepted both bearings but were slightly tighter than preferred. The ladder's Ø19.15 bore has no movement and accepts easier thumb pressure.</x:v>
       </x:c>
       <x:c r="G14" s="243" t="str">
-        <x:v>Before full link print</x:v>
+        <x:v>Complete 2026-09-02</x:v>
       </x:c>
       <x:c r="H14" s="243" t="str">
-        <x:v>$0 — use the owned bearing and existing ladder STL.</x:v>
+        <x:v>$0 — no reprint required.</x:v>
       </x:c>
       <x:c r="I14" s="243" t="str">
         <x:v>README.md lines 38–46</x:v>
@@ -5728,16 +5749,16 @@
         <x:v>RFQ &amp; Holds rows 5, 7–9</x:v>
       </x:c>
       <x:c r="E16" s="243" t="str">
-        <x:v>Request exact drawings/certificates; do not substitute rounded catalog sizes.</x:v>
+        <x:v>Complete ABS single-leg fit, assembly, wiring, and unloaded controls integration; leave the main spring unpreloaded and structural-load fixtures unused.</x:v>
       </x:c>
       <x:c r="F16" s="243" t="str">
-        <x:v>These parts set spring rate, −8° stop engagement, cartridge alignment and preload.</x:v>
+        <x:v>Geometry and wheel-clear/current-limited self-weight checks only.</x:v>
       </x:c>
       <x:c r="G16" s="243" t="str">
-        <x:v>Now for Mode A through step 6</x:v>
+        <x:v>Active now through unloaded single-leg commissioning.</x:v>
       </x:c>
       <x:c r="H16" s="243" t="str">
-        <x:v>Bundle RFQs where possible; A228 music-wire spring is acceptable for the early prototype.</x:v>
+        <x:v>No torque-arm, main-spring, ground-traction, stall/proof, drop, or human-adjacent loading in ABS.</x:v>
       </x:c>
       <x:c r="I16" s="243" t="str">
         <x:v>beni_single_leg_rig_design_record.md §9</x:v>
@@ -5844,16 +5865,16 @@
         <x:v>Conditional plus test brief steps 2–4</x:v>
       </x:c>
       <x:c r="E20" s="243" t="str">
-        <x:v>Inventory or borrow first. A normal DMM does not replace the milliohm measurement; latency needs two observable timing channels.</x:v>
+        <x:v>Use the DMM, 4-wire milliohm meter and 2-channel scope/logic tools for wiring, phase resistance, latency and the unloaded CAN soak; defer the scale and force/torque/spring instrumentation.</x:v>
       </x:c>
       <x:c r="F20" s="243" t="str">
-        <x:v>These gate torque, phase resistance, magnet-carrier TIR and &lt;8 ms loop latency.</x:v>
+        <x:v>Electrical characterization remains active; load metrology moves later.</x:v>
       </x:c>
       <x:c r="G20" s="243" t="str">
-        <x:v>Before steps 2–4</x:v>
+        <x:v>Electrical tools now; load metrology at the two-leg structural build.</x:v>
       </x:c>
       <x:c r="H20" s="243" t="str">
-        <x:v>Borrowing is the cheapest high-confidence option; buy only what cannot be borrowed.</x:v>
+        <x:v>Do not let instrument availability expand the ABS test envelope.</x:v>
       </x:c>
       <x:c r="I20" s="243" t="str">
         <x:v>fusion_brief_single_leg_rig.md §6</x:v>
@@ -5861,28 +5882,28 @@
     </x:row>
     <x:row r="21" ht="57" customHeight="1">
       <x:c r="A21" s="243" t="str">
-        <x:v>Structural release</x:v>
+        <x:v>Two-leg structural release</x:v>
       </x:c>
       <x:c r="B21" s="247" t="str">
-        <x:v>AFTER ABS FIT</x:v>
+        <x:v>DEFERRED — OWNER</x:v>
       </x:c>
       <x:c r="C21" s="243" t="str">
-        <x:v>PA6-CF and hardened 0.6 mm hotend</x:v>
+        <x:v>PA6-CF, hardened 0.6 mm hotend and material-specific coupons</x:v>
       </x:c>
       <x:c r="D21" s="243" t="str">
-        <x:v>Conditional rows 12–13</x:v>
+        <x:v>Owner scope decision 2026-09-02</x:v>
       </x:c>
       <x:c r="E21" s="243" t="str">
-        <x:v>Buy only if not already owned, after ABS geometry passes; re-run critical PA-CF fit coupons.</x:v>
+        <x:v>Finish the complete ABS single-leg integration article first; buy and calibrate PA-CF immediately before the later two-leg structural prints.</x:v>
       </x:c>
       <x:c r="F21" s="243" t="str">
-        <x:v>ABS is for unloaded fit/assembly only. Torque and spring loading require the structural material release.</x:v>
+        <x:v>ABS is valid for fit, assembly, cable routing, hand motion and wheel-clear/current-limited self-weight motor checks only. No spring characterization, ground traction, stall/proof torque or drops through ABS.</x:v>
       </x:c>
       <x:c r="G21" s="243" t="str">
-        <x:v>After ABS fit; before torque/spring loads</x:v>
+        <x:v>At two-leg structural build</x:v>
       </x:c>
       <x:c r="H21" s="243" t="str">
-        <x:v>Do not consume the PA-CF spool during fit iteration.</x:v>
+        <x:v>Defer the spool and hotend; preserve the full ABS budget for integration iteration.</x:v>
       </x:c>
       <x:c r="I21" s="243" t="str">
         <x:v>CLAUDE.md hard rule 7</x:v>
@@ -5897,8 +5918,8 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0079a13c4fcd4d70"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R405c2671a7314188"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2b392a574564cc9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20719d2288e94429"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Audit printed heat-set insert interfaces
</commit_message>
<xml_diff>
--- a/procurement/mode_a_procurement_bom_2026-08-21.xlsx
+++ b/procurement/mode_a_procurement_bom_2026-08-21.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Rc272015197034a95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order Now" sheetId="2" r:id="R0bbd23ccf2b24d1b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conditional" sheetId="3" r:id="Rac4c091a23d34bb8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ &amp; Holds" sheetId="4" r:id="R2534a57dd14544ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplier Carts" sheetId="5" r:id="R6b1daee730a846f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owned &amp; Printed" sheetId="6" r:id="R47916313bedb46e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" r:id="R9b6ff4c2aae44a11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order Links" sheetId="8" r:id="R7eaf3f4faae94f47"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status &amp; Gaps" sheetId="9" r:id="R5e722ed5af2248fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Rd364db9636ea4dcc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order Now" sheetId="2" r:id="R1d284126e4e346ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conditional" sheetId="3" r:id="R7bc753c6ff774762"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFQ &amp; Holds" sheetId="4" r:id="Rfb05944210a345ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplier Carts" sheetId="5" r:id="R5156f58c0c884f92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owned &amp; Printed" sheetId="6" r:id="Recbfcf38629e457c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" r:id="R7a8f7a8a49174c8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order Links" sheetId="8" r:id="Rd26c604b2d6c49ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status &amp; Gaps" sheetId="9" r:id="Refd93be5c4d44447"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,7 +25,7 @@
     <x:numFmt numFmtId="200" formatCode="$#,##0.00"/>
     <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
-  <x:fonts count="54">
+  <x:fonts count="59">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -334,8 +334,36 @@
       <x:color rgb="FF217346"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF17212B"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFC62828"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF33495E"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF17212B"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF33495E"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="18">
+  <x:fills count="26">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -420,6 +448,46 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F3EC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE9E7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFBFE4F3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8F3EC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE9E7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFBFE4F3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F8"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -611,7 +679,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="249">
+  <x:cellXfs count="284">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1210,6 +1278,87 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="48" fillId="18" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="54" fillId="18" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="54" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="54" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="54" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="54" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="54" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="54" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="54" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="54" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="55" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="56" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="56" fillId="20" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="56" fillId="20" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="56" fillId="20" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="56" fillId="19" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="55" fillId="19" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="54" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="54" fillId="21" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="54" fillId="21" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="54" fillId="21" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="54" fillId="22" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="55" fillId="23" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="54" fillId="23" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="57" fillId="23" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="56" fillId="24" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="55" fillId="24" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="58" fillId="24" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="58" fillId="23" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="55" fillId="23" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="54" fillId="25" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1510,7 +1659,7 @@
     <x:row r="5">
       <x:c r="A5" s="154" t="n">
         <x:f>'Order Now'!H26</x:f>
-        <x:v>146.32000000000005</x:v>
+        <x:v>140.95000000000002</x:v>
       </x:c>
       <x:c r="B5" s="155"/>
       <x:c r="C5" s="147"/>
@@ -1521,7 +1670,7 @@
       <x:c r="E5" s="157"/>
       <x:c r="F5" s="147"/>
       <x:c r="G5" s="158" t="str">
-        <x:v>4 RFQ + VERIFY + HOLD</x:v>
+        <x:v>7 OPEN GATES</x:v>
       </x:c>
       <x:c r="H5" s="159"/>
     </x:row>
@@ -1610,10 +1759,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B12" s="168" t="str">
-        <x:v>Do not buy clevis retention hardware</x:v>
+        <x:v>Close Fusion design holds before printing/buying</x:v>
       </x:c>
       <x:c r="C12" s="169" t="str">
-        <x:v>The active Fusion clevis body has no E-clip groove/cross-hole. Retention must be designed and verified through Fusion MCP first.</x:v>
+        <x:v>Correct and verify the shoulder-hub, wheel-hub and stand insert receivers, and close the clevis-pin retention scheme through Fusion MCP. The current releases must not be used for those interfaces.</x:v>
       </x:c>
       <x:c r="D12" s="147"/>
       <x:c r="E12" s="147"/>
@@ -1720,7 +1869,9 @@
       <x:c r="H20" s="171"/>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="147"/>
+      <x:c r="A21" s="147" t="str">
+        <x:v>• Heat-set scope: 14 active M3 inserts are already owned but must pass the Ø4.0 × 5.0 ABS coupon. The owned M4×8/10 inserts are too long for the thin hubs; do not force or self-tap them.</x:v>
+      </x:c>
       <x:c r="B21" s="147"/>
       <x:c r="C21" s="147"/>
       <x:c r="D21" s="147"/>
@@ -2444,38 +2595,38 @@
         <x:v>Inserts</x:v>
       </x:c>
       <x:c r="C17" s="176" t="str">
-        <x:v>M3 heat-set inserts</x:v>
+        <x:v>Voron-style M3 heat-set inserts</x:v>
       </x:c>
       <x:c r="D17" s="176" t="str">
-        <x:v>M3 brass insert, exactly 5.0 mm long; 4-pack</x:v>
+        <x:v>Owner-reported AliExpress Voron family; project receiving pocket Ø4.0 × 5.0 mm; exact order variant still to verify</x:v>
       </x:c>
       <x:c r="E17" s="176" t="str">
-        <x:v>10 pcs</x:v>
+        <x:v>14 pcs + spares</x:v>
       </x:c>
       <x:c r="F17" s="176" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G17" s="177" t="n">
-        <x:v>1.79</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H17" s="177" t="n">
         <x:f>ROUND(F17*G17,2)</x:f>
-        <x:v>5.37</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I17" s="176" t="str">
-        <x:v>PartsBuilt</x:v>
+        <x:v>Owner stock</x:v>
       </x:c>
       <x:c r="J17" s="176" t="str">
-        <x:v>PBX-TI-M3-5-4PK</x:v>
+        <x:v>AliExpress order URL / variant not recorded</x:v>
       </x:c>
       <x:c r="K17" s="178" t="str">
-        <x:v>URL tab →</x:v>
+        <x:v>OWNED — VERIFY</x:v>
       </x:c>
       <x:c r="L17" s="176" t="str">
-        <x:v>Receive 12 total. Verify length with the printed 5 mm insert coupon before installing in parts.</x:v>
+        <x:v>Count at least 14 usable inserts and fit the exact owned insert in the Ø4.0 × 5.0 ABS coupon before installing in parts.</x:v>
       </x:c>
       <x:c r="M17" s="176" t="str">
-        <x:v>Three 4-packs; small-cart shipping may dominate.</x:v>
+        <x:v>Owned; excluded from the open subtotal. Do not buy the superseded PartsBuilt packs.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="21.600000381469727" hidden="0" customHeight="1">
@@ -2489,7 +2640,7 @@
         <x:v>M4 heat/ultrasonic inserts</x:v>
       </x:c>
       <x:c r="D18" s="176" t="str">
-        <x:v>PSM Tech-Sonic brass M4, exactly 5.8 mm overall length</x:v>
+        <x:v>PSM Tech-Sonic brass M4, exactly 5.8 mm overall length; shoulder-hub candidate only</x:v>
       </x:c>
       <x:c r="E18" s="176" t="str">
         <x:v>6 pcs</x:v>
@@ -2501,7 +2652,6 @@
         <x:v>0.29</x:v>
       </x:c>
       <x:c r="H18" s="177" t="n">
-        <x:f>ROUND(F18*G18,2)</x:f>
         <x:v>1.74</x:v>
       </x:c>
       <x:c r="I18" s="176" t="str">
@@ -2514,10 +2664,10 @@
         <x:v>URL tab →</x:v>
       </x:c>
       <x:c r="L18" s="176" t="str">
-        <x:v>Do not substitute a common 6 or 8.1 mm insert; fit the 5.8 mm coupon first.</x:v>
+        <x:v>Fit an M4×5.8 coupon first. The owned M4×8/10 inserts are too long for the thin shoulder/wheel hub interfaces.</x:v>
       </x:c>
       <x:c r="M18" s="176" t="str">
-        <x:v>International/specialist shipping is not included; request a domestic shipping quote before checkout.</x:v>
+        <x:v>Shoulder-hub candidate only. Wheel-hub receiving thread remains on Fusion design hold.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
@@ -2825,7 +2975,7 @@
       <x:c r="G26" s="180"/>
       <x:c r="H26" s="180" t="n">
         <x:f>SUM(H5:H25)</x:f>
-        <x:v>146.32000000000005</x:v>
+        <x:v>140.95000000000002</x:v>
       </x:c>
       <x:c r="I26" s="179"/>
       <x:c r="J26" s="179"/>
@@ -3605,6 +3755,38 @@
         <x:v>Fusion model showing groove/cross-hole plus matching catalog hardware.</x:v>
       </x:c>
     </x:row>
+    <x:row r="11" ht="104" customHeight="1">
+      <x:c r="A11" s="275" t="str">
+        <x:v>DESIGN HOLD</x:v>
+      </x:c>
+      <x:c r="B11" s="276" t="str">
+        <x:v>Inserts</x:v>
+      </x:c>
+      <x:c r="C11" s="276" t="str">
+        <x:v>Printed threaded interfaces</x:v>
+      </x:c>
+      <x:c r="D11" s="276" t="str">
+        <x:v>Active: shoulder hub needs 6 M4 insert pockets; wheel hub needs 6 verified metal receiving threads; stand needs 5 Voron-family M3 pockets. Future chassis/carriage interfaces and the optional satellite-PCB M2 boss also require closure.</x:v>
+      </x:c>
+      <x:c r="E11" s="276" t="str">
+        <x:v>3 active parts</x:v>
+      </x:c>
+      <x:c r="F11" s="276" t="str">
+        <x:v>Restore Fusion MCP, correct each receiving interface, inspect geometry, export, and verify before printing.</x:v>
+      </x:c>
+      <x:c r="G11" s="276" t="str">
+        <x:v>Owner M3 inventory + PSM M4×5.8 shoulder candidate</x:v>
+      </x:c>
+      <x:c r="H11" s="276" t="str">
+        <x:v>Do not self-tap printed plastic or force the owned M4×8/10 inserts into thin hubs.</x:v>
+      </x:c>
+      <x:c r="I11" s="276" t="str">
+        <x:v>Current hub and stand holes are legacy/oversize for the intended inserts; the wheel-hub receiving scheme is not closed.</x:v>
+      </x:c>
+      <x:c r="J11" s="276" t="str">
+        <x:v>Fusion inspection showing pocket diameter/depth and wall/floor, plus regenerated STL and coupon/first-article fit.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:J1"/>
@@ -3827,26 +4009,26 @@
     </x:row>
     <x:row r="11" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A11" s="176" t="str">
-        <x:v>PartsBuilt</x:v>
+        <x:v>Owner stock</x:v>
       </x:c>
       <x:c r="B11" s="176" t="str">
-        <x:v>Three M3×5 mm insert 4-packs</x:v>
+        <x:v>Voron-style M3 inserts — owned; exact AliExpress variant pending</x:v>
       </x:c>
       <x:c r="C11" s="177" t="n">
         <x:f>SUMIF('Order Now'!$I$5:$I$25,A11,'Order Now'!$H$5:$H$25)</x:f>
-        <x:v>5.37</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D11" s="176" t="str">
-        <x:v>Small order; consider local pickup/combining with other exact printer parts only.</x:v>
+        <x:v>Count inventory and run the Ø4.0 × 5.0 ABS coupon before installation.</x:v>
       </x:c>
       <x:c r="E11" s="176" t="str">
-        <x:v>Shipping may exceed the item cost.</x:v>
-      </x:c>
-      <x:c r="F11" s="176" t="n">
-        <x:v>7</x:v>
+        <x:v>None — already owned.</x:v>
+      </x:c>
+      <x:c r="F11" s="176" t="str">
+        <x:v>DONE — VERIFY</x:v>
       </x:c>
       <x:c r="G11" s="176" t="str">
-        <x:v>Order or obtain the exact insert locally.</x:v>
+        <x:v>Do not order the superseded PartsBuilt packs.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
@@ -3904,7 +4086,7 @@
       <x:c r="B14" s="188"/>
       <x:c r="C14" s="189" t="n">
         <x:f>SUM(C5:C13)</x:f>
-        <x:v>146.32000000000002</x:v>
+        <x:v>140.95000000000002</x:v>
       </x:c>
       <x:c r="D14" s="188"/>
       <x:c r="E14" s="188"/>
@@ -4201,24 +4383,84 @@
         <x:v>Full-depth Ø19.10 ABS link accepts both bearings but is slightly tight; use Ø19.15 for future ABS proximal-link prints.</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="207" t="str">
-        <x:v>Deferred</x:v>
-      </x:c>
-      <x:c r="B16" s="207" t="str">
-        <x:v>Mode B rail rig</x:v>
-      </x:c>
-      <x:c r="C16" s="207" t="str">
-        <x:v>MGN12 rail/blocks, extrusion, rail hardware, quick-release pin, PU bumpers, ballast, M12 washers, M4 studs/inserts</x:v>
-      </x:c>
-      <x:c r="D16" s="207" t="str">
-        <x:v>Do not buy</x:v>
-      </x:c>
-      <x:c r="E16" s="207" t="str">
-        <x:v>beni_single_leg_rig_design_record.md §9</x:v>
-      </x:c>
-      <x:c r="F16" s="207" t="str">
-        <x:v>Re-open only after Mode A fixture and measurement gates pass.</x:v>
+    <x:row r="16" ht="60" customHeight="1">
+      <x:c r="A16" s="274" t="str">
+        <x:v>Owned — verify</x:v>
+      </x:c>
+      <x:c r="B16" s="274" t="str">
+        <x:v>Inserts</x:v>
+      </x:c>
+      <x:c r="C16" s="274" t="str">
+        <x:v>Voron-style M3 heat-set inserts</x:v>
+      </x:c>
+      <x:c r="D16" s="274" t="str">
+        <x:v>On hand; count pending</x:v>
+      </x:c>
+      <x:c r="E16" s="274" t="str">
+        <x:v>Owner-reported AliExpress purchase; exact order URL/variant not accessible</x:v>
+      </x:c>
+      <x:c r="F16" s="274" t="str">
+        <x:v>Fit the exact insert in the Ø4.0 × 5.0 ABS coupon; reserve 14 for the active build.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="60" customHeight="1">
+      <x:c r="A17" s="274" t="str">
+        <x:v>Owned</x:v>
+      </x:c>
+      <x:c r="B17" s="274" t="str">
+        <x:v>Inserts</x:v>
+      </x:c>
+      <x:c r="C17" s="274" t="str">
+        <x:v>M3 brass insert assortment</x:v>
+      </x:c>
+      <x:c r="D17" s="274" t="str">
+        <x:v>400 pcs labeled</x:v>
+      </x:c>
+      <x:c r="E17" s="274" t="str">
+        <x:v>evidence/inserts/2026-09-02_received/m3_assortment_400pc.jpg</x:v>
+      </x:c>
+      <x:c r="F17" s="274" t="str">
+        <x:v>Label dimensions identify families but do not define a CAD receiving bore; coupon-test before use.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="60" customHeight="1">
+      <x:c r="A18" s="274" t="str">
+        <x:v>Owned</x:v>
+      </x:c>
+      <x:c r="B18" s="274" t="str">
+        <x:v>Inserts</x:v>
+      </x:c>
+      <x:c r="C18" s="274" t="str">
+        <x:v>M2/M3/M4/M5 threaded insert assortment</x:v>
+      </x:c>
+      <x:c r="D18" s="274" t="str">
+        <x:v>520 pcs labeled</x:v>
+      </x:c>
+      <x:c r="E18" s="274" t="str">
+        <x:v>evidence/inserts/2026-09-02_received/m2_m3_m4_m5_assortment_520pc.jpg</x:v>
+      </x:c>
+      <x:c r="F18" s="274" t="str">
+        <x:v>M4 stock is 8/10 mm long and is not an approved substitute for the thin shoulder or wheel hub.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="60" customHeight="1">
+      <x:c r="A19" s="274" t="str">
+        <x:v>Owned — verify</x:v>
+      </x:c>
+      <x:c r="B19" s="274" t="str">
+        <x:v>Inserts</x:v>
+      </x:c>
+      <x:c r="C19" s="274" t="str">
+        <x:v>Voron-style M3 heat-set inserts</x:v>
+      </x:c>
+      <x:c r="D19" s="274" t="str">
+        <x:v>On hand; count pending</x:v>
+      </x:c>
+      <x:c r="E19" s="274" t="str">
+        <x:v>Owner-reported AliExpress purchase; exact order URL/variant not accessible</x:v>
+      </x:c>
+      <x:c r="F19" s="274" t="str">
+        <x:v>Fit the exact insert in the Ø4.0 × 5.0 ABS coupon; reserve 14 for the active build.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4650,6 +4892,66 @@
         <x:v>Ordered 2026-08-31; actual checkout total was not provided.</x:v>
       </x:c>
     </x:row>
+    <x:row r="23" ht="58" customHeight="1">
+      <x:c r="A23" s="283" t="str">
+        <x:v>Evidence</x:v>
+      </x:c>
+      <x:c r="B23" s="283" t="str">
+        <x:v>Received threaded-insert inventory</x:v>
+      </x:c>
+      <x:c r="C23" s="283" t="str">
+        <x:v>Owner has separate Voron-style M3 inserts plus labeled 400-piece M3 and 520-piece M2/M3/M4/M5 assortments</x:v>
+      </x:c>
+      <x:c r="D23" s="283" t="str">
+        <x:v>2026-09-02</x:v>
+      </x:c>
+      <x:c r="E23" s="283" t="str">
+        <x:v>/Users/neilchulani/Robots/Biped/evidence/inserts/2026-09-02_received/README.md</x:v>
+      </x:c>
+      <x:c r="F23" s="283" t="str">
+        <x:v>The exact AliExpress Voron listing/variant was not accessible; package labels alone do not define receiving-hole geometry.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="58" customHeight="1">
+      <x:c r="A24" s="283" t="str">
+        <x:v>Project</x:v>
+      </x:c>
+      <x:c r="B24" s="283" t="str">
+        <x:v>Manufacturing constraints — threaded interfaces</x:v>
+      </x:c>
+      <x:c r="C24" s="283" t="str">
+        <x:v>Canonical active/future heat-set map, quantities, approved exceptions and design holds</x:v>
+      </x:c>
+      <x:c r="D24" s="283" t="str">
+        <x:v>2026-09-02</x:v>
+      </x:c>
+      <x:c r="E24" s="283" t="str">
+        <x:v>/Users/neilchulani/Robots/Biped/MANUFACTURING_CONSTRAINTS.md</x:v>
+      </x:c>
+      <x:c r="F24" s="283" t="str">
+        <x:v>Corrected CAD/STLs remain unreleased until Fusion MCP verification.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="58" customHeight="1">
+      <x:c r="A25" s="283" t="str">
+        <x:v>Manufacturer</x:v>
+      </x:c>
+      <x:c r="B25" s="283" t="str">
+        <x:v>PSM Tech-Sonic insert catalog</x:v>
+      </x:c>
+      <x:c r="C25" s="283" t="str">
+        <x:v>M3 and M4 insert envelope, recommended receiving-hole diameters, lengths and minimum wall guidance</x:v>
+      </x:c>
+      <x:c r="D25" s="283" t="str">
+        <x:v>2026-09-02</x:v>
+      </x:c>
+      <x:c r="E25" s="283" t="str">
+        <x:v>https://psmcelada.it/?dl=5346</x:v>
+      </x:c>
+      <x:c r="F25" s="283" t="str">
+        <x:v>M4×5.8 is a shoulder-hub candidate; the wheel-hub interface still requires Fusion closure.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>
@@ -4918,19 +5220,19 @@
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="176" t="str">
-        <x:v>Order Now</x:v>
+        <x:v>Owned / verify</x:v>
       </x:c>
       <x:c r="B17" s="176" t="str">
-        <x:v>M3 heat-set inserts</x:v>
+        <x:v>Voron-style M3 heat-set inserts</x:v>
       </x:c>
       <x:c r="C17" s="176" t="str">
-        <x:v>PartsBuilt</x:v>
+        <x:v>AliExpress — owner order</x:v>
       </x:c>
       <x:c r="D17" s="192" t="str">
-        <x:v>https://partsbuilt.com/m3-heat-set-thread-insert-5mm-long-4-pack/</x:v>
+        <x:v>Owner AliExpress order URL / variant not recorded</x:v>
       </x:c>
       <x:c r="E17" s="176" t="str">
-        <x:v>Order Now row 17</x:v>
+        <x:v>Owned &amp; Printed row 16; evidence/inserts/2026-09-02_received/README.md</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
@@ -5909,6 +6211,35 @@
         <x:v>CLAUDE.md hard rule 7</x:v>
       </x:c>
     </x:row>
+    <x:row r="22" ht="112" customHeight="1">
+      <x:c r="A22" s="278" t="str">
+        <x:v>Threaded interfaces</x:v>
+      </x:c>
+      <x:c r="B22" s="282" t="str">
+        <x:v>DESIGN HOLD</x:v>
+      </x:c>
+      <x:c r="C22" s="278" t="str">
+        <x:v>Shoulder hub, wheel hub and stand insert receivers</x:v>
+      </x:c>
+      <x:c r="D22" s="278" t="str">
+        <x:v>MANUFACTURING_CONSTRAINTS.md / RFQ &amp; Holds row 11</x:v>
+      </x:c>
+      <x:c r="E22" s="278" t="str">
+        <x:v>Restore Fusion MCP; rebuild, inspect and export corrected parts. Do not print or assemble the current hub/stand/wheel-hub releases.</x:v>
+      </x:c>
+      <x:c r="F22" s="278" t="str">
+        <x:v>The proximal link and cable cover already have valid Ø4.0 × 5.0 M3 pockets. Current hub/stand/wheel receiving interfaces do not satisfy the owned insert families.</x:v>
+      </x:c>
+      <x:c r="G22" s="278" t="str">
+        <x:v>Before shoulder-to-link or wheel-rim assembly</x:v>
+      </x:c>
+      <x:c r="H22" s="278" t="str">
+        <x:v>$0 M3 purchase now; M4 shoulder candidate remains open; wheel scheme waits for CAD closure.</x:v>
+      </x:c>
+      <x:c r="I22" s="278" t="str">
+        <x:v>Insert evidence indexed 2026-09-02; corrected Fusion/STL evidence pending</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:I1"/>
@@ -5918,8 +6249,8 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2b392a574564cc9"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20719d2288e94429"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R876452d0a3dd4285"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf8ee2b37a6943a0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>